<commit_message>
Stage 8 review fixes: E-014
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/garethb_old_laptop/Commercial/Chamber_Capacity/ChamberRates_2023_v3_FINAL_final.xlsx
+++ b/output/archive/Archive/Users/garethb_old_laptop/Commercial/Chamber_Capacity/ChamberRates_2023_v3_FINAL_final.xlsx
@@ -144,7 +144,7 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>Still 885 on the list. Check with Nick before we quote the per-pull figure to the client, they have asked twice.</t>
+        <t>Check with Nicholas Hennebry before quoting the list pull charge; the client has asked twice.</t>
       </text>
     </comment>
   </commentList>
@@ -157,7 +157,7 @@
     <author>Gareth Bramwell</author>
   </authors>
   <commentList>
-    <comment ref="B3" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0" shapeId="0">
       <text>
         <t>Occupancy assumption is a guess from the spring. Don't use it without the booking log.</t>
       </text>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,21 @@
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Rates as list in 2022. Not yet agreed with Finance for the 2023 round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Westravelle Analytical Ltd, a Tarnovell company</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Working copy v3 — 18 Nov 2022; superseded</t>
         </is>
       </c>
     </row>
@@ -578,6 +593,11 @@
           <t>Topic</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Working note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -611,7 +631,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Monthly storage charge still to be agreed with Finance. Do not quote until Alice has signed it off.</t>
+          <t>Storage-month rate (GBP): not agreed. Confirm against the commercial rate record before quoting; no numeric rate entered here.</t>
         </is>
       </c>
     </row>
@@ -637,9 +657,6 @@
       <c r="B7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -655,7 +672,7 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29.3" customWidth="1" min="1" max="1"/>
+    <col width="31.4" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -689,7 +706,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Pull charge</t>
+          <t>Pull events (not a GBP cost)</t>
         </is>
       </c>
       <c r="B4" s="2">

</xml_diff>